<commit_message>
Add single-period backtest command and relabel walk-forward folds
backtest.py forecasts any period already in the file using only earlier
information, scores every model against the actual weights and exports a
per-stock table. Falls back to naive with a clear message when no training
rows exist before the base period, and offers an explicit in-sample switch.
Walk-forward columns are now named by the period being forecast, and the
volatility feature can be switched off via Config.use_vol.
</commit_message>
<xml_diff>
--- a/output/forecast_next_period.xlsx
+++ b/output/forecast_next_period.xlsx
@@ -65292,12 +65292,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Dec-24</t>
+          <t>Dec-25</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Dec-25</t>
+          <t>Aug-26</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">

</xml_diff>